<commit_message>
Bookings example: a duplicate in the manual sheet, caught and rejected
The manual Excel sheet gets TC022, TC020 again under another title, as a sheet
that grew over the years has. check names it as a repeat of TC020 and the
reviewer rejects it. The README's check now shows what check says right after
the import, before the review, and the guide lists the rule.
</commit_message>
<xml_diff>
--- a/examples/bookings-team/existing/manual_cases.xlsx
+++ b/examples/bookings-team/existing/manual_cases.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -556,6 +556,48 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC022</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Refund status after a late cancel</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>A booking made two days ago</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1. Cancel the booking 2. Open its refund status</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>The status is no_refund and the amount is 0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>AC-5</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>refund</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>